<commit_message>
Enhancements on script generation and added new featrure test daat generation
</commit_message>
<xml_diff>
--- a/output/Test_Cases_collection/TC02 - Login with Invalid Username.xlsx
+++ b/output/Test_Cases_collection/TC02 - Login with Invalid Username.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="29">
   <si>
     <t>Test Case Name</t>
   </si>
@@ -52,28 +52,46 @@
     <t>3</t>
   </si>
   <si>
-    <t>Launch the application and open `https://www.saucedemo.com/`.</t>
-  </si>
-  <si>
-    <t>Enter `invalid_user` in the "user-name" field.</t>
-  </si>
-  <si>
-    <t>Enter `secret_sauce` in the "password" field.</t>
-  </si>
-  <si>
-    <t>Click on "login-button".</t>
-  </si>
-  <si>
-    <t>The login page is displayed with username and password fields.</t>
-  </si>
-  <si>
-    <t>The username is entered successfully.</t>
-  </si>
-  <si>
-    <t>The password is entered successfully.</t>
-  </si>
-  <si>
-    <t>An error message is displayed: "Epic sadface: Username and password do not match any user in this service."</t>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Launch the application and open [https://www.saucedemo.com/]</t>
+  </si>
+  <si>
+    <t>Click on "user-name"</t>
+  </si>
+  <si>
+    <t>Enter "invalid_user" in the "user-name" field</t>
+  </si>
+  <si>
+    <t>Click on "password"</t>
+  </si>
+  <si>
+    <t>Enter "secret_sauce" in the "password" field</t>
+  </si>
+  <si>
+    <t>Click on "login-button"</t>
+  </si>
+  <si>
+    <t>Application is launched successfully</t>
+  </si>
+  <si>
+    <t>"user-name" field is focused</t>
+  </si>
+  <si>
+    <t>Username is entered successfully</t>
+  </si>
+  <si>
+    <t>"password" field is focused</t>
+  </si>
+  <si>
+    <t>Password is entered successfully</t>
+  </si>
+  <si>
+    <t>Error message "Epic sadface: Username and password do not match any user in this service" is displayed</t>
   </si>
   <si>
     <t>New</t>
@@ -440,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -474,19 +492,19 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="G2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -497,16 +515,16 @@
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -517,16 +535,16 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -537,16 +555,56 @@
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
         <v>19</v>
       </c>
-      <c r="E5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" t="s">
-        <v>21</v>
+      <c r="D7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
screenshot handles, few more bug fixes
</commit_message>
<xml_diff>
--- a/output/Test_Cases_collection/TC02 - Login with Invalid Username.xlsx
+++ b/output/Test_Cases_collection/TC02 - Login with Invalid Username.xlsx
@@ -52,28 +52,28 @@
     <t>3</t>
   </si>
   <si>
-    <t>Launch the application and open `https://www.saucedemo.com/`.</t>
-  </si>
-  <si>
-    <t>Enter "invalid_user" in the "user-name" field.</t>
-  </si>
-  <si>
-    <t>Enter "secret_sauce" in the "password" field.</t>
-  </si>
-  <si>
-    <t>Click on "login-button".</t>
-  </si>
-  <si>
-    <t>The login page is displayed with username and password fields.</t>
-  </si>
-  <si>
-    <t>The username is entered successfully.</t>
-  </si>
-  <si>
-    <t>The password is entered successfully.</t>
-  </si>
-  <si>
-    <t>An error message is displayed: "Epic sadface: Username and password do not match any user in this service."</t>
+    <t>Launch the application and open [https://www.saucedemo.com/]</t>
+  </si>
+  <si>
+    <t>Enter "invalid_user" in "user-name" field</t>
+  </si>
+  <si>
+    <t>Enter "secret_sauce" in "password" field</t>
+  </si>
+  <si>
+    <t>Click on "login-button"</t>
+  </si>
+  <si>
+    <t>Application is launched, and the login page is displayed</t>
+  </si>
+  <si>
+    <t>Username is entered successfully</t>
+  </si>
+  <si>
+    <t>Password is entered successfully</t>
+  </si>
+  <si>
+    <t>Error message "Epic sadface: Username and password do not match any user in this service" is displayed</t>
   </si>
   <si>
     <t>New</t>

</xml_diff>